<commit_message>
Align candidate rules and review workbook with approved R8 mapping
</commit_message>
<xml_diff>
--- a/docs/architecture/business-rules/evidence/业务规则审阅表.xlsx
+++ b/docs/architecture/business-rules/evidence/业务规则审阅表.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="业务规则" sheetId="1" r:id="R4658bc89181747a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="操作与影响" sheetId="2" r:id="R25a7d5284d0e46bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本次变化" sheetId="3" r:id="Rd567221f8da04d90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="业务规则" sheetId="1" r:id="Rfb0ae9989cb44588"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="操作与影响" sheetId="2" r:id="R6bc3b8ba263e41a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本次变化" sheetId="3" r:id="R614fed6677774b6f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -125,8 +125,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OperationsReview" displayName="OperationsReview" ref="A5:E22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:E22"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OperationsReview" displayName="OperationsReview" ref="A5:E24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:E24"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="业务名称"/>
     <x:tableColumn id="2" name="改变什么"/>
@@ -368,7 +368,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="str">
-        <x:v>审阅数据SHA256：e346d967f661c9bbf72acb78844d8a6ae15fe76458f8502e2393b5e3b2a9a221</x:v>
+        <x:v>审阅数据SHA256：966b195c679952d3d542658be3c661ad2a7e328473ac6d0f27f1f08be190c459</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -378,12 +378,12 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>A包候选 · candidate-2026-10-15-compact1 · 不切生产</x:v>
+        <x:v>A包候选 · candidate-2026-10-16-r8 · 不切生产</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>现有业务政策摘要；最终对齐等待映射批准。技术组合由测试核验，黄色列保留审阅意见。</x:v>
+        <x:v>已合并R8业务政策摘要；候选未接生产。业务条件保留，黄色列保留审阅意见。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="36" hidden="0" customHeight="1">
@@ -428,7 +428,7 @@
         <x:v>稳定审阅键</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="6" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A6" s="5" t="str">
         <x:v>燃料直接含碳量</x:v>
       </x:c>
@@ -440,8 +440,10 @@
         <x:v>MASS: tC/t; VOLUME: tC/10^4Nm3</x:v>
       </x:c>
       <x:c r="D6" s="5" t="str">
-        <x:v>实测值
-适用：对象类别=目录对象或自定义或历史身份未确认</x:v>
+        <x:v>计算值 / 实测值
+适用：对象类别=目录对象或自定义
+实测值
+适用：对象类别=历史身份未确认</x:v>
       </x:c>
       <x:c r="E6" s="5" t="str">
         <x:v>实测值
@@ -453,13 +455,16 @@
       </x:c>
       <x:c r="G6" s="5" t="str">
         <x:v>数值待核验，来源可填写/选择；资格或适用性条件未满足，暂不可直接采用
-适用：对象类别=目录对象或自定义或历史身份未确认，当前来源=缺省值或计算值
+适用：对象类别=目录对象或自定义，当前来源=缺省值；
+对象类别=历史身份未确认，当前来源=缺省值或计算值
+数值可填写/选择，来源可填写/选择
+适用：对象类别=目录对象或自定义，当前来源=计算值或实测值
 数值可填写/选择，来源只读
-适用：对象类别=目录对象或自定义或历史身份未确认，当前来源=实测值</x:v>
+适用：对象类别=历史身份未确认，当前来源=实测值</x:v>
       </x:c>
       <x:c r="H6" s="5" t="str"/>
       <x:c r="I6" s="5" t="str">
-        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；并行复核中，最终对齐待批准）
+        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；依据已合并的PR48 Mapping）
 已批准软件决定及当前HANDOFF；机器定义仅执行表达，不另解释标准。</x:v>
       </x:c>
       <x:c r="J6" s="5" t="str"/>
@@ -467,7 +472,7 @@
       <x:c r="L6" s="8" t="str"/>
       <x:c r="M6" s="8" t="str"/>
       <x:c r="N6" s="9" t="str">
-        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-15-compact1|fuel.direct_carbon|SUMMARY</x:v>
+        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-16-r8|fuel.direct_carbon|SUMMARY</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="264" hidden="0" customHeight="1">
@@ -482,9 +487,9 @@
         <x:v>MASS: GJ/t; VOLUME: GJ/10⁴Nm³; HEAT: GJ/GJ when supplied</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
-        <x:v>缺省值 / 计算值 / 实测值
+        <x:v>缺省值 / 实测值
 适用：对象类别=目录对象，绑定资格=来源登记已核验，须匹配精确登记组合（26项）
-计算值 / 实测值
+实测值
 适用：对象类别=自定义或目录对象，绑定资格=无适用绑定
 待核验
 适用：对象类别=历史身份未确认，绑定资格=待核验</x:v>
@@ -492,7 +497,7 @@
       <x:c r="E7" s="5" t="str">
         <x:v>缺省值
 适用：对象类别=目录对象，绑定资格=来源登记已核验，须匹配精确登记组合（26项）
-无自动默认
+实测值
 适用：对象类别=自定义或目录对象，绑定资格=无适用绑定
 待核验
 适用：对象类别=历史身份未确认，绑定资格=待核验</x:v>
@@ -520,7 +525,7 @@
       </x:c>
       <x:c r="H7" s="5" t="str"/>
       <x:c r="I7" s="5" t="str">
-        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；并行复核中，最终对齐待批准）
+        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；依据已合并的PR48 Mapping）
 已批准软件决定及当前HANDOFF；机器定义仅执行表达，不另解释标准。</x:v>
       </x:c>
       <x:c r="J7" s="5" t="str"/>
@@ -528,7 +533,7 @@
       <x:c r="L7" s="8" t="str"/>
       <x:c r="M7" s="8" t="str"/>
       <x:c r="N7" s="9" t="str">
-        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-15-compact1|fuel.lhv|SUMMARY</x:v>
+        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-16-r8|fuel.lhv|SUMMARY</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="264" hidden="0" customHeight="1">
@@ -542,9 +547,9 @@
         <x:v>tC/GJ (HEAT path)</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:v>缺省值 / 计算值 / 实测值
+        <x:v>缺省值 / 实测值
 适用：对象类别=目录对象，绑定资格=来源登记已核验，须匹配精确登记组合（26项）
-计算值 / 实测值
+实测值
 适用：对象类别=自定义或目录对象，绑定资格=无适用绑定
 待核验
 适用：对象类别=历史身份未确认，绑定资格=待核验</x:v>
@@ -552,7 +557,7 @@
       <x:c r="E8" s="5" t="str">
         <x:v>缺省值
 适用：对象类别=目录对象，绑定资格=来源登记已核验，须匹配精确登记组合（26项）
-无自动默认
+实测值
 适用：对象类别=自定义或目录对象，绑定资格=无适用绑定
 待核验
 适用：对象类别=历史身份未确认，绑定资格=待核验</x:v>
@@ -580,7 +585,7 @@
       </x:c>
       <x:c r="H8" s="5" t="str"/>
       <x:c r="I8" s="5" t="str">
-        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；并行复核中，最终对齐待批准）
+        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；依据已合并的PR48 Mapping）
 已批准软件决定及当前HANDOFF；机器定义仅执行表达，不另解释标准。</x:v>
       </x:c>
       <x:c r="J8" s="5" t="str"/>
@@ -588,7 +593,7 @@
       <x:c r="L8" s="8" t="str"/>
       <x:c r="M8" s="8" t="str"/>
       <x:c r="N8" s="9" t="str">
-        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-15-compact1|fuel.fch|SUMMARY</x:v>
+        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-16-r8|fuel.fch|SUMMARY</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="303.6000061035156" hidden="0" customHeight="1">
@@ -641,7 +646,7 @@
       </x:c>
       <x:c r="H9" s="5" t="str"/>
       <x:c r="I9" s="5" t="str">
-        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；并行复核中，最终对齐待批准）
+        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；依据已合并的PR48 Mapping）
 已批准软件决定及当前HANDOFF；机器定义仅执行表达，不另解释标准。</x:v>
       </x:c>
       <x:c r="J9" s="5" t="str"/>
@@ -649,10 +654,10 @@
       <x:c r="L9" s="8" t="str"/>
       <x:c r="M9" s="8" t="str"/>
       <x:c r="N9" s="9" t="str">
-        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-15-compact1|fuel.oxidation|SUMMARY</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="105.5999984741211" hidden="0" customHeight="1">
+        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-16-r8|fuel.oxidation|SUMMARY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="132" hidden="0" customHeight="1">
       <x:c r="A10" s="5" t="str">
         <x:v>原料固定碳含量</x:v>
       </x:c>
@@ -670,8 +675,12 @@
         <x:v>%</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
-        <x:v>实测值
-适用：绑定资格=无适用绑定</x:v>
+        <x:v>实测值 / 计算值
+适用：共同条件：绑定资格=无适用绑定；且满足以下任一情形：
+当前来源=实测值；
+当前来源=计算值，已定义物料换算路径=已批准收到基换算（仍核必要数值/基准）
+无合法来源
+适用：绑定资格=无适用绑定，当前来源=缺省值</x:v>
       </x:c>
       <x:c r="E10" s="5" t="str">
         <x:v>实测值
@@ -683,13 +692,15 @@
       </x:c>
       <x:c r="G10" s="5" t="str">
         <x:v>数值待核验，来源可填写/选择；资格或适用性条件未满足，暂不可直接采用
-适用：绑定资格=无适用绑定，当前来源=缺省值或计算值
-数值可填写/选择，来源只读
-适用：绑定资格=无适用绑定，当前来源=实测值</x:v>
+适用：绑定资格=无适用绑定，当前来源=缺省值
+数值可填写/选择，来源可填写/选择
+适用：共同条件：绑定资格=无适用绑定；且满足以下任一情形：
+当前来源=实测值；
+当前来源=计算值，已定义物料换算路径=已批准收到基换算（仍核必要数值/基准）</x:v>
       </x:c>
       <x:c r="H10" s="5" t="str"/>
       <x:c r="I10" s="5" t="str">
-        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；并行复核中，最终对齐待批准）
+        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；依据已合并的PR48 Mapping）
 已批准软件决定及当前HANDOFF；机器定义仅执行表达，不另解释标准。</x:v>
       </x:c>
       <x:c r="J10" s="5" t="str"/>
@@ -697,10 +708,10 @@
       <x:c r="L10" s="8" t="str"/>
       <x:c r="M10" s="8" t="str"/>
       <x:c r="N10" s="9" t="str">
-        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-15-compact1|material.fixed_carbon|SUMMARY</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-16-r8|material.fixed_carbon|SUMMARY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="132" hidden="0" customHeight="1">
       <x:c r="A11" s="5" t="str">
         <x:v>原料挥发分含量</x:v>
       </x:c>
@@ -715,8 +726,12 @@
         <x:v>%</x:v>
       </x:c>
       <x:c r="D11" s="5" t="str">
-        <x:v>实测值
-适用：绑定资格=无适用绑定</x:v>
+        <x:v>实测值 / 计算值
+适用：共同条件：绑定资格=无适用绑定；且满足以下任一情形：
+当前来源=实测值；
+当前来源=计算值，已定义物料换算路径=已批准收到基换算（仍核必要数值/基准）
+无合法来源
+适用：绑定资格=无适用绑定，当前来源=缺省值</x:v>
       </x:c>
       <x:c r="E11" s="5" t="str">
         <x:v>实测值
@@ -728,13 +743,15 @@
       </x:c>
       <x:c r="G11" s="5" t="str">
         <x:v>数值待核验，来源可填写/选择；资格或适用性条件未满足，暂不可直接采用
-适用：绑定资格=无适用绑定，当前来源=缺省值或计算值
-数值可填写/选择，来源只读
-适用：绑定资格=无适用绑定，当前来源=实测值</x:v>
+适用：绑定资格=无适用绑定，当前来源=缺省值
+数值可填写/选择，来源可填写/选择
+适用：共同条件：绑定资格=无适用绑定；且满足以下任一情形：
+当前来源=实测值；
+当前来源=计算值，已定义物料换算路径=已批准收到基换算（仍核必要数值/基准）</x:v>
       </x:c>
       <x:c r="H11" s="5" t="str"/>
       <x:c r="I11" s="5" t="str">
-        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；并行复核中，最终对齐待批准）
+        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；依据已合并的PR48 Mapping）
 已批准软件决定及当前HANDOFF；机器定义仅执行表达，不另解释标准。</x:v>
       </x:c>
       <x:c r="J11" s="5" t="str"/>
@@ -742,7 +759,7 @@
       <x:c r="L11" s="8" t="str"/>
       <x:c r="M11" s="8" t="str"/>
       <x:c r="N11" s="9" t="str">
-        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-15-compact1|material.volatile_matter|SUMMARY</x:v>
+        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-16-r8|material.volatile_matter|SUMMARY</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="356.3999938964844" hidden="0" customHeight="1">
@@ -757,53 +774,53 @@
       </x:c>
       <x:c r="D12" s="5" t="str">
         <x:v>缺省值 / 实测值
-适用：绑定资格=来源登记已核验，本实例组分数=1，须匹配精确登记组合（1项）
+适用：绑定资格=来源登记已核验，本批有效组分数=1，须匹配精确登记组合（1项）
 实测值
 适用：共同条件：绑定资格=无适用绑定；且满足以下任一情形：
-本实例组分数=1；
-本实例组分数≥2
+本批有效组分数=1；
+本批有效组分数≥2
 待核验
-适用：绑定资格=待核验，本实例组分数≥1</x:v>
+适用：绑定资格=待核验，本批有效组分数≥1</x:v>
       </x:c>
       <x:c r="E12" s="5" t="str">
         <x:v>缺省值
-适用：绑定资格=来源登记已核验，本实例组分数=1，须匹配精确登记组合（1项）
+适用：绑定资格=来源登记已核验，本批有效组分数=1，须匹配精确登记组合（1项）
 实测值
 适用：共同条件：绑定资格=无适用绑定；且满足以下任一情形：
-本实例组分数=1；
-本实例组分数≥2
+本批有效组分数=1；
+本批有效组分数≥2
 待核验
-适用：绑定资格=待核验，本实例组分数≥1</x:v>
+适用：绑定资格=待核验，本批有效组分数≥1</x:v>
       </x:c>
       <x:c r="F12" s="5" t="str">
         <x:v>缺省路径按适用精确绑定从参数与因子库读取
-适用：绑定资格=来源登记已核验，当前来源=缺省值，本实例组分数=1，须匹配精确登记组合（1项）
+适用：绑定资格=来源登记已核验，当前来源=缺省值，本批有效组分数=1，须匹配精确登记组合（1项）
 不自动填写数值；按来源与输入要求填写
-适用：绑定资格=无适用绑定，当前来源=缺省值，本实例组分数=1；
-绑定资格=无适用绑定，当前来源=缺省值，本实例组分数≥2；
+适用：绑定资格=无适用绑定，当前来源=缺省值，本批有效组分数=1；
+绑定资格=无适用绑定，当前来源=缺省值，本批有效组分数≥2；
 当前来源=实测值或计算值
 适用性未完成核对，暂不自动填写
-适用：绑定资格=待核验，当前来源=缺省值，本实例组分数≥1</x:v>
+适用：绑定资格=待核验，当前来源=缺省值，本批有效组分数≥1</x:v>
       </x:c>
       <x:c r="G12" s="5" t="str">
         <x:v>数值只读，来源可填写/选择
-适用：绑定资格=来源登记已核验，当前来源=缺省值，本实例组分数=1，须匹配精确登记组合（1项）
+适用：绑定资格=来源登记已核验，当前来源=缺省值，本批有效组分数=1，须匹配精确登记组合（1项）
 数值待核验，来源可填写/选择；资格或适用性条件未满足，暂不可直接采用
-适用：绑定资格=来源登记已核验，当前来源=计算值，本实例组分数=1，须匹配精确登记组合（1项）；
-绑定资格=无适用绑定，当前来源=缺省值或计算值，本实例组分数=1；
-绑定资格=无适用绑定，当前来源=缺省值或计算值，本实例组分数≥2
+适用：绑定资格=来源登记已核验，当前来源=计算值，本批有效组分数=1，须匹配精确登记组合（1项）；
+绑定资格=无适用绑定，当前来源=缺省值或计算值，本批有效组分数=1；
+绑定资格=无适用绑定，当前来源=缺省值或计算值，本批有效组分数≥2
 数值可填写/选择，来源可填写/选择
-适用：绑定资格=来源登记已核验，当前来源=实测值，本实例组分数=1，须匹配精确登记组合（1项）
+适用：绑定资格=来源登记已核验，当前来源=实测值，本批有效组分数=1，须匹配精确登记组合（1项）
 数值可填写/选择，来源只读
 适用：共同条件：绑定资格=无适用绑定，当前来源=实测值；且满足以下任一情形：
-本实例组分数=1；
-本实例组分数≥2
+本批有效组分数=1；
+本批有效组分数≥2
 数值待核验，来源待核验；资格或适用性条件未满足，暂不可直接采用
-适用：绑定资格=待核验，当前来源=缺省值或计算值或实测值，本实例组分数≥1</x:v>
+适用：绑定资格=待核验，当前来源=缺省值或计算值或实测值，本批有效组分数≥1</x:v>
       </x:c>
       <x:c r="H12" s="5" t="str"/>
       <x:c r="I12" s="5" t="str">
-        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；并行复核中，最终对齐待批准）
+        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；依据已合并的PR48 Mapping）
 已批准软件决定及当前HANDOFF；机器定义仅执行表达，不另解释标准。</x:v>
       </x:c>
       <x:c r="J12" s="5" t="str"/>
@@ -811,7 +828,7 @@
       <x:c r="L12" s="8" t="str"/>
       <x:c r="M12" s="8" t="str"/>
       <x:c r="N12" s="9" t="str">
-        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-15-compact1|fgd.ratio|SUMMARY</x:v>
+        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-16-r8|fgd.ratio|SUMMARY</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="237.60000610351562" hidden="0" customHeight="1">
@@ -862,7 +879,7 @@
       </x:c>
       <x:c r="H13" s="5" t="str"/>
       <x:c r="I13" s="5" t="str">
-        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；并行复核中，最终对齐待批准）
+        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；依据已合并的PR48 Mapping）
 已批准软件决定及当前HANDOFF；机器定义仅执行表达，不另解释标准。</x:v>
       </x:c>
       <x:c r="J13" s="5" t="str"/>
@@ -870,7 +887,7 @@
       <x:c r="L13" s="8" t="str"/>
       <x:c r="M13" s="8" t="str"/>
       <x:c r="N13" s="9" t="str">
-        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-15-compact1|fgd.factor|SUMMARY</x:v>
+        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-16-r8|fgd.factor|SUMMARY</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="277.20001220703125" hidden="0" customHeight="1">
@@ -923,7 +940,7 @@
       </x:c>
       <x:c r="H14" s="5" t="str"/>
       <x:c r="I14" s="5" t="str">
-        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；并行复核中，最终对齐待批准）
+        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；依据已合并的PR48 Mapping）
 已批准软件决定及当前HANDOFF；机器定义仅执行表达，不另解释标准。</x:v>
       </x:c>
       <x:c r="J14" s="5" t="str"/>
@@ -931,10 +948,10 @@
       <x:c r="L14" s="8" t="str"/>
       <x:c r="M14" s="8" t="str"/>
       <x:c r="N14" s="9" t="str">
-        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-15-compact1|fgd.conversion|SUMMARY</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="1768.800048828125" hidden="0" customHeight="1">
+        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-16-r8|fgd.conversion|SUMMARY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="1412.4000244140625" hidden="0" customHeight="1">
       <x:c r="A15" s="5" t="str">
         <x:v>购入/输出电力因子</x:v>
       </x:c>
@@ -950,17 +967,17 @@
 适用：共同条件：对象类别=目录对象，绑定资格=来源登记已核验；且满足以下任一情形：
 因子路径=目录表1，方向=购入，电力属性=常规电力，来源表=1，须匹配精确登记组合（1项）；
 因子路径=目录表1，方向=输出，来源表=1，须匹配精确登记组合（1项）；
+因子路径=目录表2，方向=购入，电力属性=常规电力，来源表=2，须匹配精确登记组合（7项）；
+因子路径=目录表2，方向=输出，来源表=2，须匹配精确登记组合（7项）；
 因子路径=目录表3，方向=购入，电力属性=常规电力，来源表=3，须匹配精确登记组合（30项）；
 因子路径=目录表3，方向=输出，来源表=3，须匹配精确登记组合（30项）；
+因子路径=目录表4，方向=购入，电力属性=常规电力，来源表=4，须匹配精确登记组合（1项）；
+因子路径=目录表4，方向=输出，来源表=4，须匹配精确登记组合（1项）；
+因子路径=目录表5，方向=购入，电力属性=化石，来源表=5，须匹配精确登记组合（1项）；
+因子路径=目录表5，方向=输出，来源表=5，须匹配精确登记组合（1项）；
 因子路径=非化石购电零排放，方向=购入，电力属性=非化石，须匹配精确登记组合（1项）
 待核验
-适用：对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表2，方向=购入，电力属性=常规电力，来源表=2，须匹配精确登记组合（7项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表2，方向=输出，来源表=2，须匹配精确登记组合（7项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表4，方向=购入，电力属性=常规电力，来源表=4，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表4，方向=输出，来源表=4，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表5，方向=购入，电力属性=化石，来源表=5，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表5，方向=输出，来源表=5，须匹配精确登记组合（1项）；
-因子路径=供电单位实测，方向=购入或输出；
+适用：因子路径=供电单位实测，方向=购入或输出；
 因子路径=企业实测，方向=购入或输出；
 因子路径=企业计算，方向=购入或输出；
 因子路径=目录表1，方向=购入或输出，绑定资格=无适用绑定；
@@ -969,25 +986,29 @@
 因子路径=目录表4，方向=购入或输出，绑定资格=无适用绑定；
 因子路径=目录表5，方向=购入或输出，绑定资格=无适用绑定；
 因子路径=非化石购电零排放，方向=购入，绑定资格=无适用绑定
+本路径无需选择来源类别；不得冒用缺省/计算/实测
+适用：共同条件：因子路径=库外自行填写（输入方式，非来源类别）；且满足以下任一情形：
+方向=购入，电力属性=常规电力或化石；
+方向=输出
 无合法来源
-适用：因子路径=任意覆盖路径（现有候选未开放），方向=购入或输出</x:v>
+适用：因子路径=库外自行填写（输入方式，非来源类别），方向=购入，电力属性=非化石</x:v>
       </x:c>
       <x:c r="E15" s="5" t="str">
         <x:v>缺省值
 适用：共同条件：对象类别=目录对象，绑定资格=来源登记已核验；且满足以下任一情形：
 因子路径=目录表1，方向=购入，电力属性=常规电力，来源表=1，须匹配精确登记组合（1项）；
 因子路径=目录表1，方向=输出，来源表=1，须匹配精确登记组合（1项）；
+因子路径=目录表2，方向=购入，电力属性=常规电力，来源表=2，须匹配精确登记组合（7项）；
+因子路径=目录表2，方向=输出，来源表=2，须匹配精确登记组合（7项）；
 因子路径=目录表3，方向=购入，电力属性=常规电力，来源表=3，须匹配精确登记组合（30项）；
 因子路径=目录表3，方向=输出，来源表=3，须匹配精确登记组合（30项）；
+因子路径=目录表4，方向=购入，电力属性=常规电力，来源表=4，须匹配精确登记组合（1项）；
+因子路径=目录表4，方向=输出，来源表=4，须匹配精确登记组合（1项）；
+因子路径=目录表5，方向=购入，电力属性=化石，来源表=5，须匹配精确登记组合（1项）；
+因子路径=目录表5，方向=输出，来源表=5，须匹配精确登记组合（1项）；
 因子路径=非化石购电零排放，方向=购入，电力属性=非化石，须匹配精确登记组合（1项）
 待核验
-适用：对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表2，方向=购入，电力属性=常规电力，来源表=2，须匹配精确登记组合（7项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表2，方向=输出，来源表=2，须匹配精确登记组合（7项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表4，方向=购入，电力属性=常规电力，来源表=4，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表4，方向=输出，来源表=4，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表5，方向=购入，电力属性=化石，来源表=5，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表5，方向=输出，来源表=5，须匹配精确登记组合（1项）；
-因子路径=供电单位实测，方向=购入或输出；
+适用：因子路径=供电单位实测，方向=购入或输出；
 因子路径=企业实测，方向=购入或输出；
 因子路径=企业计算，方向=购入或输出；
 因子路径=目录表1，方向=购入或输出，绑定资格=无适用绑定；
@@ -997,45 +1018,32 @@
 因子路径=目录表5，方向=购入或输出，绑定资格=无适用绑定；
 因子路径=非化石购电零排放，方向=购入，绑定资格=无适用绑定
 无自动默认
-适用：因子路径=任意覆盖路径（现有候选未开放），方向=购入或输出</x:v>
+适用：共同条件：因子路径=库外自行填写（输入方式，非来源类别）；且满足以下任一情形：
+方向=购入，电力属性=常规电力或化石或非化石；
+方向=输出</x:v>
       </x:c>
       <x:c r="F15" s="5" t="str">
         <x:v>缺省路径按适用精确绑定从参数与因子库读取
-适用：共同条件：对象类别=目录对象，绑定资格=来源登记已核验，当前来源=缺省值；且满足以下任一情形：
-因子路径=目录表1，方向=购入，电力属性=常规电力，来源表=1，须匹配精确登记组合（1项）；
-因子路径=目录表1，方向=输出，来源表=1，须匹配精确登记组合（1项）；
-因子路径=目录表3，方向=购入，电力属性=常规电力，来源表=3，须匹配精确登记组合（30项）；
-因子路径=目录表3，方向=输出，来源表=3，须匹配精确登记组合（30项）；
-因子路径=非化石购电零排放，方向=购入，电力属性=非化石，须匹配精确登记组合（1项）
-适用性未完成核对，暂不自动填写
-适用：共同条件：当前来源=缺省值；且满足以下任一情形：
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表2，方向=购入，电力属性=常规电力，来源表=2，须匹配精确登记组合（7项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表2，方向=输出，来源表=2，须匹配精确登记组合（7项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表4，方向=购入，电力属性=常规电力，来源表=4，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表4，方向=输出，来源表=4，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表5，方向=购入，电力属性=化石，来源表=5，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表5，方向=输出，来源表=5，须匹配精确登记组合（1项）；
-因子路径=目录表1，方向=购入或输出，绑定资格=无适用绑定；
-因子路径=目录表2，方向=购入或输出，绑定资格=无适用绑定；
-因子路径=目录表3，方向=购入或输出，绑定资格=无适用绑定；
-因子路径=目录表4，方向=购入或输出，绑定资格=无适用绑定；
-因子路径=目录表5，方向=购入或输出，绑定资格=无适用绑定；
-因子路径=非化石购电零排放，方向=购入，绑定资格=无适用绑定
+适用：共同条件：对象类别=目录对象，绑定资格=来源登记已核验；且满足以下任一情形：
+因子路径=目录表1，方向=购入，电力属性=常规电力，来源表=1，当前来源=缺省值，须匹配精确登记组合（1项）；
+因子路径=目录表1，方向=输出，来源表=1，当前来源=缺省值，须匹配精确登记组合（1项）；
+因子路径=目录表2，方向=购入，电力属性=常规电力，来源表=2，当前来源=缺省值或计算值或实测值，须匹配精确登记组合（7项）；
+因子路径=目录表2，方向=输出，来源表=2，当前来源=缺省值或计算值或实测值，须匹配精确登记组合（7项）；
+因子路径=目录表3，方向=购入，电力属性=常规电力，来源表=3，当前来源=缺省值，须匹配精确登记组合（30项）；
+因子路径=目录表3，方向=输出，来源表=3，当前来源=缺省值，须匹配精确登记组合（30项）；
+因子路径=目录表4，方向=购入，电力属性=常规电力，来源表=4，当前来源=缺省值或计算值或实测值，须匹配精确登记组合（1项）；
+因子路径=目录表4，方向=输出，来源表=4，当前来源=缺省值或计算值或实测值，须匹配精确登记组合（1项）；
+因子路径=目录表5，方向=购入，电力属性=化石，来源表=5，当前来源=缺省值或计算值或实测值，须匹配精确登记组合（1项）；
+因子路径=目录表5，方向=输出，来源表=5，当前来源=缺省值或计算值或实测值，须匹配精确登记组合（1项）；
+因子路径=非化石购电零排放，方向=购入，电力属性=非化石，当前来源=缺省值，须匹配精确登记组合（1项）
 不自动填写数值；按来源与输入要求填写
 适用：因子路径=供电单位实测，方向=购入或输出，绑定资格=待核验，当前来源=实测值；
 因子路径=企业实测，方向=购入或输出，绑定资格=待核验，当前来源=实测值；
 因子路径=企业计算，方向=购入或输出，绑定资格=待核验，当前来源=计算值；
-因子路径=任意覆盖路径（现有候选未开放），方向=购入或输出，当前来源=实测值或缺省值或计算值；
 对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表1，方向=购入，电力属性=常规电力，来源表=1，当前来源=计算值或实测值，须匹配精确登记组合（1项）；
 对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表1，方向=输出，来源表=1，当前来源=计算值或实测值，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表2，方向=购入，电力属性=常规电力，来源表=2，当前来源=计算值或实测值，须匹配精确登记组合（7项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表2，方向=输出，来源表=2，当前来源=计算值或实测值，须匹配精确登记组合（7项）；
 对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表3，方向=购入，电力属性=常规电力，来源表=3，当前来源=计算值或实测值，须匹配精确登记组合（30项）；
 对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表3，方向=输出，来源表=3，当前来源=计算值或实测值，须匹配精确登记组合（30项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表4，方向=购入，电力属性=常规电力，来源表=4，当前来源=计算值或实测值，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表4，方向=输出，来源表=4，当前来源=计算值或实测值，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表5，方向=购入，电力属性=化石，来源表=5，当前来源=计算值或实测值，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表5，方向=输出，来源表=5，当前来源=计算值或实测值，须匹配精确登记组合（1项）；
 对象类别=目录对象，绑定资格=来源登记已核验，因子路径=非化石购电零排放，方向=购入，电力属性=非化石，当前来源=计算值或实测值，须匹配精确登记组合（1项）；
 因子路径=供电单位实测，方向=购入或输出，当前来源=缺省值或计算值；
 因子路径=企业实测，方向=购入或输出，当前来源=缺省值或计算值；
@@ -1045,46 +1053,66 @@
 因子路径=目录表3，方向=购入或输出，绑定资格=无适用绑定，当前来源=计算值或实测值；
 因子路径=目录表4，方向=购入或输出，绑定资格=无适用绑定，当前来源=计算值或实测值；
 因子路径=目录表5，方向=购入或输出，绑定资格=无适用绑定，当前来源=计算值或实测值；
-因子路径=非化石购电零排放，方向=购入，绑定资格=无适用绑定，当前来源=计算值或实测值</x:v>
+因子路径=非化石购电零排放，方向=购入，绑定资格=无适用绑定，当前来源=计算值或实测值；
+因子路径=库外自行填写（输入方式，非来源类别），方向=购入，电力属性=常规电力或化石或非化石；
+因子路径=库外自行填写（输入方式，非来源类别），方向=输出
+适用性未完成核对，暂不自动填写
+适用：共同条件：绑定资格=无适用绑定，当前来源=缺省值；且满足以下任一情形：
+因子路径=目录表1，方向=购入或输出；
+因子路径=目录表2，方向=购入或输出；
+因子路径=目录表3，方向=购入或输出；
+因子路径=目录表4，方向=购入或输出；
+因子路径=目录表5，方向=购入或输出；
+因子路径=非化石购电零排放，方向=购入</x:v>
       </x:c>
       <x:c r="G15" s="5" t="str">
         <x:v>数值只读，来源只读
-适用：共同条件：对象类别=目录对象，绑定资格=来源登记已核验，当前来源=缺省值；且满足以下任一情形：
-因子路径=目录表1，方向=购入，电力属性=常规电力，来源表=1，须匹配精确登记组合（1项）；
-因子路径=目录表1，方向=输出，来源表=1，须匹配精确登记组合（1项）；
-因子路径=目录表3，方向=购入，电力属性=常规电力，来源表=3，须匹配精确登记组合（30项）；
-因子路径=目录表3，方向=输出，来源表=3，须匹配精确登记组合（30项）；
-因子路径=非化石购电零排放，方向=购入，电力属性=非化石，须匹配精确登记组合（1项）
+适用：共同条件：当前来源=缺省值；且满足以下任一情形：
+对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表1，方向=购入，电力属性=常规电力，来源表=1，须匹配精确登记组合（1项）；
+对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表1，方向=输出，来源表=1，须匹配精确登记组合（1项）；
+对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表2，方向=购入，电力属性=常规电力，来源表=2，须匹配精确登记组合（7项）；
+对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表2，方向=输出，来源表=2，须匹配精确登记组合（7项）；
+对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表3，方向=购入，电力属性=常规电力，来源表=3，须匹配精确登记组合（30项）；
+对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表3，方向=输出，来源表=3，须匹配精确登记组合（30项）；
+对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表4，方向=购入，电力属性=常规电力，来源表=4，须匹配精确登记组合（1项）；
+对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表4，方向=输出，来源表=4，须匹配精确登记组合（1项）；
+对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表5，方向=购入，电力属性=化石，来源表=5，须匹配精确登记组合（1项）；
+对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表5，方向=输出，来源表=5，须匹配精确登记组合（1项）；
+对象类别=目录对象，绑定资格=来源登记已核验，因子路径=非化石购电零排放，方向=购入，电力属性=非化石，须匹配精确登记组合（1项）；
+因子路径=目录表1，方向=购入或输出，绑定资格=无适用绑定
 数值待核验，来源可填写/选择；资格或适用性条件未满足，暂不可直接采用
 适用：共同条件：对象类别=目录对象，绑定资格=来源登记已核验，当前来源=计算值或实测值；且满足以下任一情形：
 因子路径=目录表1，方向=购入，电力属性=常规电力，来源表=1，须匹配精确登记组合（1项）；
 因子路径=目录表1，方向=输出，来源表=1，须匹配精确登记组合（1项）；
+因子路径=目录表2，方向=购入，电力属性=常规电力，来源表=2，须匹配精确登记组合（7项）；
+因子路径=目录表2，方向=输出，来源表=2，须匹配精确登记组合（7项）；
 因子路径=目录表3，方向=购入，电力属性=常规电力，来源表=3，须匹配精确登记组合（30项）；
 因子路径=目录表3，方向=输出，来源表=3，须匹配精确登记组合（30项）；
+因子路径=目录表4，方向=购入，电力属性=常规电力，来源表=4，须匹配精确登记组合（1项）；
+因子路径=目录表4，方向=输出，来源表=4，须匹配精确登记组合（1项）；
+因子路径=目录表5，方向=购入，电力属性=化石，来源表=5，须匹配精确登记组合（1项）；
+因子路径=目录表5，方向=输出，来源表=5，须匹配精确登记组合（1项）；
 因子路径=非化石购电零排放，方向=购入，电力属性=非化石，须匹配精确登记组合（1项）
 数值待核验，来源待核验；资格或适用性条件未满足，暂不可直接采用
-适用：共同条件：当前来源=缺省值或计算值或实测值；且满足以下任一情形：
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表2，方向=购入，电力属性=常规电力，来源表=2，须匹配精确登记组合（7项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表2，方向=输出，来源表=2，须匹配精确登记组合（7项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表4，方向=购入，电力属性=常规电力，来源表=4，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表4，方向=输出，来源表=4，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表5，方向=购入，电力属性=化石，来源表=5，须匹配精确登记组合（1项）；
-对象类别=目录对象，绑定资格=来源登记已核验，因子路径=目录表5，方向=输出，来源表=5，须匹配精确登记组合（1项）；
-因子路径=供电单位实测，方向=购入或输出；
-因子路径=企业实测，方向=购入或输出；
-因子路径=企业计算，方向=购入或输出；
-因子路径=目录表1，方向=购入或输出，绑定资格=无适用绑定；
-因子路径=目录表2，方向=购入或输出，绑定资格=无适用绑定；
-因子路径=目录表3，方向=购入或输出，绑定资格=无适用绑定；
-因子路径=目录表4，方向=购入或输出，绑定资格=无适用绑定；
-因子路径=目录表5，方向=购入或输出，绑定资格=无适用绑定；
-因子路径=非化石购电零排放，方向=购入，绑定资格=无适用绑定
-数值不适用，来源只读
-适用：因子路径=任意覆盖路径（现有候选未开放），方向=购入或输出，当前来源=缺省值或计算值或实测值</x:v>
+适用：因子路径=供电单位实测，方向=购入或输出，当前来源=缺省值或计算值或实测值；
+因子路径=企业实测，方向=购入或输出，当前来源=缺省值或计算值或实测值；
+因子路径=企业计算，方向=购入或输出，当前来源=缺省值或计算值或实测值；
+因子路径=目录表1，方向=购入或输出，绑定资格=无适用绑定，当前来源=计算值或实测值；
+因子路径=目录表2，方向=购入或输出，绑定资格=无适用绑定，当前来源=缺省值或计算值或实测值；
+因子路径=目录表3，方向=购入或输出，绑定资格=无适用绑定，当前来源=缺省值或计算值或实测值；
+因子路径=目录表4，方向=购入或输出，绑定资格=无适用绑定，当前来源=缺省值或计算值或实测值；
+因子路径=目录表5，方向=购入或输出，绑定资格=无适用绑定，当前来源=缺省值或计算值或实测值；
+因子路径=非化石购电零排放，方向=购入，绑定资格=无适用绑定，当前来源=缺省值或计算值或实测值
+数值可填写/选择，来源不适用
+适用：共同条件：因子路径=库外自行填写（输入方式，非来源类别）；且满足以下任一情形：
+方向=购入，电力属性=常规电力或化石；
+方向=输出
+数值只读，来源不适用
+适用：因子路径=库外自行填写（输入方式，非来源类别），方向=购入，电力属性=非化石</x:v>
       </x:c>
       <x:c r="H15" s="5" t="str"/>
       <x:c r="I15" s="5" t="str">
-        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；并行复核中，最终对齐待批准）
+        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；依据已合并的PR48 Mapping）
 已批准软件决定及当前HANDOFF；机器定义仅执行表达，不另解释标准。</x:v>
       </x:c>
       <x:c r="J15" s="5" t="str"/>
@@ -1092,7 +1120,7 @@
       <x:c r="L15" s="8" t="str"/>
       <x:c r="M15" s="8" t="str"/>
       <x:c r="N15" s="9" t="str">
-        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-15-compact1|electricity.factor|SUMMARY</x:v>
+        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-16-r8|electricity.factor|SUMMARY</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="303.6000061035156" hidden="0" customHeight="1">
@@ -1146,7 +1174,7 @@
       </x:c>
       <x:c r="H16" s="5" t="str"/>
       <x:c r="I16" s="5" t="str">
-        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；并行复核中，最终对齐待批准）
+        <x:v>specs/carbon_accounting/GB_T_32151_34_2024_MAPPING.md §8/§9（对应mapping_refs；依据已合并的PR48 Mapping）
 已批准软件决定及当前HANDOFF；机器定义仅执行表达，不另解释标准。</x:v>
       </x:c>
       <x:c r="J16" s="5" t="str"/>
@@ -1154,7 +1182,7 @@
       <x:c r="L16" s="8" t="str"/>
       <x:c r="M16" s="8" t="str"/>
       <x:c r="N16" s="9" t="str">
-        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-15-compact1|heat.factor|SUMMARY</x:v>
+        <x:v>field|qz.carbon_accounting.industry.gbt_32151_34_2024|candidate-2026-10-16-r8|heat.factor|SUMMARY</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1165,7 +1193,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48991c5195474a1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re58d5eaaaada469f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1191,7 +1219,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="str">
-        <x:v>审阅数据SHA256：e346d967f661c9bbf72acb78844d8a6ae15fe76458f8502e2393b5e3b2a9a221</x:v>
+        <x:v>审阅数据SHA256：966b195c679952d3d542658be3c661ad2a7e328473ac6d0f27f1f08be190c459</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -1201,12 +1229,12 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>A包候选 · candidate-2026-10-15-compact1 · 不切生产</x:v>
+        <x:v>A包候选 · candidate-2026-10-16-r8 · 不切生产</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>现有业务政策摘要；最终对齐等待映射批准。技术组合由测试核验，黄色列保留审阅意见。</x:v>
+        <x:v>已合并R8业务政策摘要；候选未接生产。业务条件保留，黄色列保留审阅意见。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="36" hidden="0" customHeight="1">
@@ -1264,7 +1292,7 @@
       <x:c r="H6" s="8" t="str"/>
       <x:c r="I6" s="8" t="str"/>
       <x:c r="J6" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|initialize_new_accounting</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|initialize_new_accounting</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -1289,7 +1317,7 @@
       <x:c r="H7" s="8" t="str"/>
       <x:c r="I7" s="8" t="str"/>
       <x:c r="J7" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|edit_name_draft</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|edit_name_draft</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -1314,7 +1342,7 @@
       <x:c r="H8" s="8" t="str"/>
       <x:c r="I8" s="8" t="str"/>
       <x:c r="J8" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|confirm_same_catalog_identity</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|confirm_same_catalog_identity</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="92.4000015258789" hidden="0" customHeight="1">
@@ -1342,7 +1370,7 @@
       <x:c r="H9" s="8" t="str"/>
       <x:c r="I9" s="8" t="str"/>
       <x:c r="J9" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|switch_catalog_identity</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|switch_catalog_identity</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1367,7 +1395,7 @@
       <x:c r="H10" s="8" t="str"/>
       <x:c r="I10" s="8" t="str"/>
       <x:c r="J10" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|switch_source_isolated_draft</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|switch_source_isolated_draft</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -1392,7 +1420,7 @@
       <x:c r="H11" s="8" t="str"/>
       <x:c r="I11" s="8" t="str"/>
       <x:c r="J11" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|change_fuel_path_unit</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|change_fuel_path_unit</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -1415,7 +1443,7 @@
       <x:c r="H12" s="8" t="str"/>
       <x:c r="I12" s="8" t="str"/>
       <x:c r="J12" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|edit_repeat_groups</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|edit_repeat_groups</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -1438,7 +1466,7 @@
       <x:c r="H13" s="8" t="str"/>
       <x:c r="I13" s="8" t="str"/>
       <x:c r="J13" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|restore_without_default_init</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|restore_without_default_init</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1461,7 +1489,7 @@
       <x:c r="H14" s="8" t="str"/>
       <x:c r="I14" s="8" t="str"/>
       <x:c r="J14" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|download_approved_template</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|download_approved_template</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="66" hidden="0" customHeight="1">
@@ -1485,7 +1513,7 @@
       <x:c r="H15" s="8" t="str"/>
       <x:c r="I15" s="8" t="str"/>
       <x:c r="J15" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|project_upgrade_cancel</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|project_upgrade_cancel</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -1509,7 +1537,7 @@
       <x:c r="H16" s="8" t="str"/>
       <x:c r="I16" s="8" t="str"/>
       <x:c r="J16" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|excel_preview</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|excel_preview</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1532,18 +1560,21 @@
       <x:c r="H17" s="8" t="str"/>
       <x:c r="I17" s="8" t="str"/>
       <x:c r="J17" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|save_restore_project</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|save_restore_project</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A18" s="5" t="str">
         <x:v>正式核算并追加不可变正式记录</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>一条COMPLETED或COMPLETED_WITH_WARNINGS正式正式记录</x:v>
+        <x:v>每次成功核算新增一条COMPLETED或COMPLETED_WITH_WARNINGS正式正式记录，并冻结本次输入、结果、参数快照、规则与证据
+若外部CO₂已纳入且有效，另冻结补充合计；ES、EI、ET保持不变</x:v>
       </x:c>
       <x:c r="C18" s="5" t="str">
-        <x:v>既有正式记录及其快照</x:v>
+        <x:v>既有正式记录及其快照
+材料附件缺失/未审核只提醒；必要值、数量基准、方法和身份仍校验
+未提供外部补充不表示活动不存在，旧正式记录不补造补充值</x:v>
       </x:c>
       <x:c r="D18" s="5" t="str">
         <x:v>仅新增正式记录</x:v>
@@ -1554,18 +1585,21 @@
       <x:c r="H18" s="8" t="str"/>
       <x:c r="I18" s="8" t="str"/>
       <x:c r="J18" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|formal_calculation_append_record</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|formal_calculation_append_record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A19" s="5" t="str">
         <x:v>从冻结正式记录构建并导出Word报告</x:v>
       </x:c>
       <x:c r="B19" s="5" t="str">
-        <x:v>本次导出的Word文档及导出审计事件</x:v>
+        <x:v>生成本次Word文档及导出审计事件
+存在时单独展示正式记录中已冻结的外部补充合计，不重算</x:v>
       </x:c>
       <x:c r="C19" s="5" t="str">
-        <x:v>冻结正式记录输入、结果、参数与规则快照</x:v>
+        <x:v>冻结正式记录输入、结果、参数与规则快照
+ES/EI/ET与独立冻结的外部补充合计各自原样保留
+旧正式记录缺少补充字段时不合成零值或改写历史</x:v>
       </x:c>
       <x:c r="D19" s="5" t="str">
         <x:v>只新增导出产物/审计记录，不改正式记录</x:v>
@@ -1576,7 +1610,7 @@
       <x:c r="H19" s="8" t="str"/>
       <x:c r="I19" s="8" t="str"/>
       <x:c r="J19" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|read_record_render_word</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|read_record_render_word</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1598,32 +1632,34 @@
       <x:c r="H20" s="8" t="str"/>
       <x:c r="I20" s="8" t="str"/>
       <x:c r="J20" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|soft_delete_record</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="118.80000305175781" hidden="0" customHeight="1">
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|soft_delete_record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="132" hidden="0" customHeight="1">
       <x:c r="A21" s="5" t="str">
         <x:v>按来源条件解析参数默认、来源与读写锁</x:v>
       </x:c>
       <x:c r="B21" s="5" t="str">
-        <x:v>所选字段的默认来源、合法来源与锁定状态</x:v>
+        <x:v>所选字段的默认来源、合法来源与锁定状态
+电力库外值的实际采用值与可选来源说明；不改变参数库绑定或参数库值</x:v>
       </x:c>
       <x:c r="C21" s="5" t="str">
-        <x:v>参数库正式参数值与绑定真源</x:v>
+        <x:v>参数库正式参数值与绑定真源
+Issue014已批准的库外输入产品选择与其专业适用关系OPEN状态相互独立</x:v>
       </x:c>
       <x:c r="D21" s="5" t="str">
         <x:v>仅确定该字段在当前核算上下文下的输入状态</x:v>
       </x:c>
       <x:c r="E21" s="5" t="str">
-        <x:v>Issue014 supply-unit measured/enterprise calculated paths remain PENDING.
-Electricity Table 2/4/5 applicability remains PENDING until PR46@77d36a1/Issue010 is integrated; source registration review_status is recorded separately.</x:v>
+        <x:v>Candidate-only: the updated decisions are not yet wired into the production parameter Resolver/UI.
+Issue014 professional applicability remains OPEN only for supply-unit measured / enterprise-calculated paths; the out-of-catalog product choice is approved.</x:v>
       </x:c>
       <x:c r="F21" s="5" t="str"/>
       <x:c r="G21" s="8" t="str"/>
       <x:c r="H21" s="8" t="str"/>
       <x:c r="I21" s="8" t="str"/>
       <x:c r="J21" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|resolve_parameter_source</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|resolve_parameter_source</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="79.19999694824219" hidden="0" customHeight="1">
@@ -1651,18 +1687,70 @@
       <x:c r="H22" s="8" t="str"/>
       <x:c r="I22" s="8" t="str"/>
       <x:c r="J22" s="9" t="str">
-        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|toggle_emission_source</x:v>
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|toggle_emission_source</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A23" s="5" t="str">
+        <x:v>录入并冻结外部CO₂补充值</x:v>
+      </x:c>
+      <x:c r="B23" s="5" t="str">
+        <x:v>仅改变外部补充的纳入状态及其独立冻结合计
+外部补充合计不并入、不覆盖ES、EI或ET</x:v>
+      </x:c>
+      <x:c r="C23" s="5" t="str">
+        <x:v>GB/T 32151.34原ES、EI、ET及其正式正式记录
+其他行业和范围外上下游运输算法不进入本操作
+未纳入状态不推断外部活动不存在</x:v>
+      </x:c>
+      <x:c r="D23" s="5" t="str">
+        <x:v>仅本次未保存输入的结果；成功核算后补充值与合计随正式记录冻结</x:v>
+      </x:c>
+      <x:c r="E23" s="5" t="str">
+        <x:v>Candidate-only operation boundary; production input, 正式记录, Excel/Word integration and formal acceptance remain future work.</x:v>
+      </x:c>
+      <x:c r="F23" s="5" t="str"/>
+      <x:c r="G23" s="8" t="str"/>
+      <x:c r="H23" s="8" t="str"/>
+      <x:c r="I23" s="8" t="str"/>
+      <x:c r="J23" s="9" t="str">
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|capture_external_co2_supplement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A24" s="5" t="str">
+        <x:v>蒸汽自动焓路径候选边界</x:v>
+      </x:c>
+      <x:c r="B24" s="5" t="str">
+        <x:v>仅描述未来自动焓候选路径及其边界，不改变本次生产计算</x:v>
+      </x:c>
+      <x:c r="C24" s="5" t="str">
+        <x:v>合法独立已知焓与自动求焓路径分开
+历史正式记录及其已保存的焓来源/数值</x:v>
+      </x:c>
+      <x:c r="D24" s="5" t="str">
+        <x:v>自动路径输入状态仅影响依赖自动焓的未保存结果</x:v>
+      </x:c>
+      <x:c r="E24" s="5" t="str">
+        <x:v>Candidate-only: no dependency installation or production implementation; property subprofile, fixed dependency version, independent numeric references and Conformance remain outstanding.</x:v>
+      </x:c>
+      <x:c r="F24" s="5" t="str"/>
+      <x:c r="G24" s="8" t="str"/>
+      <x:c r="H24" s="8" t="str"/>
+      <x:c r="I24" s="8" t="str"/>
+      <x:c r="J24" s="9" t="str">
+        <x:v>operation|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|resolve_steam_enthalpy</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="H6:H22">
+    <x:dataValidation type="list" sqref="H6:H24">
       <x:formula1>"待处理,已落实,需决定,保留"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62413fff775a4e65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b7d4a2c0c534ec4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1688,7 +1776,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="str">
-        <x:v>审阅数据SHA256：e346d967f661c9bbf72acb78844d8a6ae15fe76458f8502e2393b5e3b2a9a221</x:v>
+        <x:v>审阅数据SHA256：966b195c679952d3d542658be3c661ad2a7e328473ac6d0f27f1f08be190c459</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -1698,12 +1786,12 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>A包候选 · candidate-2026-10-15-compact1 · 不切生产</x:v>
+        <x:v>A包候选 · candidate-2026-10-16-r8 · 不切生产</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>现有业务政策摘要；最终对齐等待映射批准。技术组合由测试核验，黄色列保留审阅意见。</x:v>
+        <x:v>已合并R8业务政策摘要；候选未接生产。业务条件保留，黄色列保留审阅意见。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="36" hidden="0" customHeight="1">
@@ -1757,7 +1845,7 @@
       <x:c r="H6" s="8" t="str"/>
       <x:c r="I6" s="8" t="str"/>
       <x:c r="J6" s="9" t="str">
-        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|review.change.candidate_bundle</x:v>
+        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|review.change.candidate_bundle</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="79.19999694824219" hidden="0" customHeight="1">
@@ -1781,10 +1869,10 @@
       <x:c r="H7" s="8" t="str"/>
       <x:c r="I7" s="8" t="str"/>
       <x:c r="J7" s="9" t="str">
-        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|review.change.fixed_c01_adoption</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="105.5999984741211" hidden="0" customHeight="1">
+        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|review.change.fixed_c01_adoption</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A8" s="5" t="str">
         <x:v>ELECTRICITY_SOURCE_QUALIFICATION</x:v>
       </x:c>
@@ -1792,20 +1880,21 @@
         <x:v>main G05 snapshot records source-rule facts but does not encode the full PR46/Issue010 regional and five-parameter applicability policy.</x:v>
       </x:c>
       <x:c r="C8" s="5" t="str">
-        <x:v>A separates source-binding registration review from .34 software applicability: main Table 1 and verified Table 3 paths remain qualified; Table 2/4/5 paths and Issue014 supply-unit measured/enterprise calculated paths remain PENDING.</x:v>
+        <x:v>R8按分路径表达电力来源资格与软件选择：默认库内，允许库外输入，适用性/年份为非阻断提醒，来源说明选填；不得借用参数库身份或自动标记MEASURED。供电单位实测/企业测算适用关系另保持Issue014专业OPEN。</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:v>现存候选仍保留原严格适用分支。本轮只做收缩，不接管生产；Owner关于库外电力因子、非阻断核实提醒和来源选填的最新决定已批准，见HANDOFF，待映射任务协调后再落实，不再请求重复批准。来源登记VERIFIED与软件适用性继续分开。</x:v>
+        <x:v>同步已批准的Issue014库外输入产品选择与R8 Mapping；产品决定不等于专业适用性结论，来源登记状态也不代替软件来源资格。</x:v>
       </x:c>
       <x:c r="E8" s="5" t="str">
-        <x:v>既有PR46/Issue010目录组合与最新Owner外部因子决定等待映射/实现对齐；不是Owner产品选择未定。</x:v>
+        <x:v>Candidate-only; production Resolver/UI integration remains future work.
+Issue014 professional review remains OPEN only for supply-unit measured / enterprise-calculated applicability; the out-of-catalog product choice is approved.</x:v>
       </x:c>
       <x:c r="F8" s="5" t="str"/>
       <x:c r="G8" s="8" t="str"/>
       <x:c r="H8" s="8" t="str"/>
       <x:c r="I8" s="8" t="str"/>
       <x:c r="J8" s="9" t="str">
-        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|review.change.electricity_applicability</x:v>
+        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|review.change.electricity_applicability</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="79.19999694824219" hidden="0" customHeight="1">
@@ -1829,7 +1918,7 @@
       <x:c r="H9" s="8" t="str"/>
       <x:c r="I9" s="8" t="str"/>
       <x:c r="J9" s="9" t="str">
-        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|review.change.same_identity_confirmation</x:v>
+        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|review.change.same_identity_confirmation</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="118.80000305175781" hidden="0" customHeight="1">
@@ -1843,17 +1932,17 @@
         <x:v>Industry 11个稳定参数目标字段增加初始来源属性与逐条件政策：仅NEW_SELECTION、CONFIRMED_IDENTITY_CHANGE、RESELECT_AFTER_LEAVE触发；terminal结果是单一FIXED来源、NONE或PENDING。技术/legacy镜像字段显式NONE；数值默认、来源资格、锁定保持独立。</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
-        <x:v>落实V1.2 §7.1的首次默认来源行为并与数值参数库默认分开。custom/unbound LHV/FCh不自动选来源；无匹配碳酸盐EF1按Owner已批准决定默认MEASURED、数值默认为NONE并由用户填写；氧化率/直接碳/材料/FGD/heat按已核现行政策明确；表2/4/5和Issue014仍PENDING。</x:v>
+        <x:v>按R8 Mapping逐字段登记新对象首次来源，不将数值参数库默认与业务来源混为一谈。无目录匹配碳酸盐EF的实测来源决定及必要数值校验按已批准口径执行；电力库外输入产品选择已批准，Issue014仅保留特定供电单位实测/企业测算路径的专业OPEN。</x:v>
       </x:c>
       <x:c r="E10" s="5" t="str">
-        <x:v>A只定义候选初始来源语义，不实现GUI/Excel/Domain状态机或更改历史Project。</x:v>
+        <x:v>A候选仅记录初始来源语义，不实现GUI/Excel/Domain状态机或修改历史Project。</x:v>
       </x:c>
       <x:c r="F10" s="5" t="str"/>
       <x:c r="G10" s="8" t="str"/>
       <x:c r="H10" s="8" t="str"/>
       <x:c r="I10" s="8" t="str"/>
       <x:c r="J10" s="9" t="str">
-        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|review.change.initial_source_policy</x:v>
+        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|review.change.initial_source_policy</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="79.19999694824219" hidden="0" customHeight="1">
@@ -1877,7 +1966,7 @@
       <x:c r="H11" s="8" t="str"/>
       <x:c r="I11" s="8" t="str"/>
       <x:c r="J11" s="9" t="str">
-        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|review.change.channel_units</x:v>
+        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|review.change.channel_units</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -1901,32 +1990,32 @@
       <x:c r="H12" s="8" t="str"/>
       <x:c r="I12" s="8" t="str"/>
       <x:c r="J12" s="9" t="str">
-        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|review.change.source_involvement_semantics</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="79.19999694824219" hidden="0" customHeight="1">
+        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|review.change.source_involvement_semantics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A13" s="5" t="str">
-        <x:v>MAPPING_REVIEW_PENDING</x:v>
+        <x:v>MAPPING_R8_ALIGNMENT</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
         <x:v>原A出口要求完整内部字段盘点和上千技术组合审阅。</x:v>
       </x:c>
       <x:c r="C13" s="5" t="str">
-        <x:v>默认只展示业务政策、关键操作与变化；关联已有Mapping ID。最终规则一致性等待并行映射核验和Owner批准。</x:v>
+        <x:v>本候选按已完成的R8 Mapping和Issue 015/016/017批准决定同步关键操作；Mapping承担标准业务含义权威，候选只保留跨入口政策和操作摘要。</x:v>
       </x:c>
       <x:c r="D13" s="5" t="str">
-        <x:v>不把代码现状升格为标准，不新增平行规范，不根据旧A PASS宣称新规则最终就绪。</x:v>
+        <x:v>R8 Mapping已完成本轮最终整理；本次只是同步候选审阅表达，不产生第二套Mapping，不改已批准V1.2历史文件，也不自动采用到生产。</x:v>
       </x:c>
       <x:c r="E13" s="5" t="str">
-        <x:v>并行映射复核及Owner最终批准；本步不改Mapping/标准问题台账、不接生产。
-烟气焚烧P04A来源政策未纳入现有11项候选，不得套用fuel.*；等待映射核验明确。</x:v>
+        <x:v>Candidate-only; production implementation, numerical/Word acceptance and formal adoption remain separate later work.
+P04A烟气焚烧专属来源政策未纳入本压缩候选；生产接入应按R8逐字段确认，不沿用fuel.*来源政策。</x:v>
       </x:c>
       <x:c r="F13" s="5" t="str"/>
       <x:c r="G13" s="8" t="str"/>
       <x:c r="H13" s="8" t="str"/>
       <x:c r="I13" s="8" t="str"/>
       <x:c r="J13" s="9" t="str">
-        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-15-compact1|review.change.mapping_alignment</x:v>
+        <x:v>change|qz.carbon_accounting.software_policy|candidate-2026-10-16-r8|review.change.mapping_alignment</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1937,7 +2026,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06633c7b91334946"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a844c60b6e34e1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>